<commit_message>
Update AI-Specific Model analysis
</commit_message>
<xml_diff>
--- a/statistics/RQ3/AI_Specific_Model.xlsx
+++ b/statistics/RQ3/AI_Specific_Model.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sunkexin/PycharmProjects/AIReviewerAnalysis(Online)/statistics/RQ3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sunkexin/Desktop/AI Review 实证/新RQ3（2）/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DB1CD98-FA2A-C74F-8849-61C7FDDC1BBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{176EA828-B276-E04D-BE58-056EFD9EB1AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12740" yWindow="1620" windowWidth="27640" windowHeight="16860" activeTab="6" xr2:uid="{BC2FD56B-C4BC-CE47-9803-954B0AA227BC}"/>
+    <workbookView xWindow="13880" yWindow="1140" windowWidth="27640" windowHeight="16860" activeTab="6" xr2:uid="{BC2FD56B-C4BC-CE47-9803-954B0AA227BC}"/>
   </bookViews>
   <sheets>
     <sheet name="SHAP Summary" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="92">
   <si>
     <t>source</t>
   </si>
@@ -142,27 +142,15 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Trigger_auto</t>
-  </si>
-  <si>
     <t>Source_anc95/ChatGPT-CodeReview</t>
   </si>
   <si>
     <t>Source_coderabbitai/ai-pr-reviewer</t>
   </si>
   <si>
-    <t>Model_gpt-3.5</t>
-  </si>
-  <si>
     <t>Source_mattzcarey/code-review-gpt</t>
   </si>
   <si>
-    <t>Model_gpt-4</t>
-  </si>
-  <si>
-    <t>Trigger_manual</t>
-  </si>
-  <si>
     <t>🔹 Group: textual</t>
   </si>
   <si>
@@ -190,9 +178,6 @@
     <t>🔹 Group: repo</t>
   </si>
   <si>
-    <t>Trigger_auto:</t>
-  </si>
-  <si>
     <t>Is_File_Level_Action:</t>
   </si>
   <si>
@@ -268,22 +253,13 @@
     <t>Comment_Dels:</t>
   </si>
   <si>
-    <t>Model_gpt-3.5:</t>
-  </si>
-  <si>
     <t>Source_mattzcarey/code-review-gpt:</t>
   </si>
   <si>
     <t>Has_Inline_Code:</t>
   </si>
   <si>
-    <t>Model_gpt-4:</t>
-  </si>
-  <si>
     <t>Is_Programming_File:</t>
-  </si>
-  <si>
-    <t>Trigger_manual:</t>
   </si>
   <si>
     <t>Author_Is_Anonymous:</t>
@@ -323,61 +299,18 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Average result of 5-fold cross-validation
-</t>
-    </r>
+    <t>Average result of 5-fold cross-validation
+🎯 Average Final Accuracy: 0.9171
+🎯 Average Macro F1: 0.6472</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Apple Color Emoji"/>
         <family val="4"/>
-      </rPr>
-      <t>🎯</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="4"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Average Final Accuracy: 0.9171
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Apple Color Emoji"/>
-        <family val="4"/>
-      </rPr>
-      <t>🎯</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="4"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Average Macro F1: 0.6470</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Apple Color Emoji"/>
-        <family val="4"/>
-        <charset val="134"/>
       </rPr>
       <t>🌍</t>
     </r>
@@ -390,28 +323,36 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> Global Average Feature Importance (mean(|SHAP|) over all features):0.0059</t>
+      <t xml:space="preserve"> 全局平均特征重要性 (mean(|SHAP|)): 0.0064</t>
     </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Modification Feature (12): P |φ|=0.0746; μ|φ|=0.0068</t>
+    <t>Model_Is_GPT4:</t>
+  </si>
+  <si>
+    <t>Trigger_Is_Manual:</t>
+  </si>
+  <si>
+    <t>Model_Is_GPT4</t>
+  </si>
+  <si>
+    <t>Trigger_Is_Manual</t>
+  </si>
+  <si>
+    <t>Repository Feature (3): P |φ|=0.0203; μ|φ|=0.0068</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Comment Feature (10): P |φ|=0.0691; μ|φ|=0.0063</t>
+    <t>Modification Feature (12): P |φ|=0.0767; μ|φ|=0.0064</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Repository Feature (3): P |φ|=0.0203; μ|φ|=0.0048</t>
+    <t>Source Feature (7): P |φ|=0.0418; μ|φ|=0.0060</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Source Feature (9): P |φ|=0.0434; μ|φ|=0.0062</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Comment_Adds</t>
+    <t>Comment Feature (11): P |φ|=0.0709; μ|φ|=0.0064</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -423,7 +364,7 @@
     <numFmt numFmtId="176" formatCode="0.0000_ "/>
     <numFmt numFmtId="177" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -457,13 +398,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Apple Color Emoji"/>
-      <family val="4"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <b/>
       <i/>
       <sz val="12"/>
@@ -480,7 +414,7 @@
       <family val="4"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -490,6 +424,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -523,7 +463,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -539,7 +479,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -554,19 +494,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -576,6 +510,15 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -900,10 +843,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="72" customHeight="1">
-      <c r="A1" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="B1" s="16"/>
+      <c r="A1" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="14"/>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
@@ -920,10 +863,10 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>7.46E-2</v>
+        <v>6.7999999999999996E-3</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -931,23 +874,23 @@
         <v>27</v>
       </c>
       <c r="B6" s="2">
-        <v>6.9099999999999995E-2</v>
+        <v>6.4000000000000003E-3</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B7" s="2">
-        <v>4.3400000000000001E-2</v>
+        <v>6.4000000000000003E-3</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B8" s="2">
-        <v>2.0299999999999999E-2</v>
+        <v>6.0000000000000001E-3</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -965,10 +908,10 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B12" s="2">
-        <v>6.7999999999999996E-3</v>
+        <v>7.6700000000000004E-2</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -976,34 +919,34 @@
         <v>27</v>
       </c>
       <c r="B13" s="2">
-        <v>6.3E-3</v>
+        <v>7.0900000000000005E-2</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="B14" s="2">
-        <v>6.1999999999999998E-3</v>
+        <v>4.1799999999999997E-2</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B15" s="2">
-        <v>4.7999999999999996E-3</v>
+        <v>2.0299999999999999E-2</v>
       </c>
     </row>
     <row r="17" spans="1:2">
-      <c r="A17" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="B17" s="16"/>
+      <c r="A17" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B17" s="14"/>
     </row>
     <row r="18" spans="1:2" ht="39" customHeight="1">
-      <c r="A18" s="16"/>
-      <c r="B18" s="16"/>
+      <c r="A18" s="14"/>
+      <c r="B18" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1017,7 +960,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B83602CB-4BF0-8842-8535-6C17BF0753D9}">
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
@@ -1027,10 +970,10 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>30</v>
@@ -1044,13 +987,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C2" s="6">
-        <v>1.9800000000000002E-2</v>
+        <v>2.12E-2</v>
       </c>
       <c r="D2" s="8">
-        <v>-0.67190000000000005</v>
+        <v>-0.6744</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1058,13 +1001,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C3" s="6">
-        <v>1.44E-2</v>
+        <v>1.77E-2</v>
       </c>
       <c r="D3" s="8">
-        <v>0.91449999999999998</v>
+        <v>0.92230000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1072,13 +1015,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C4" s="6">
-        <v>1.21E-2</v>
+        <v>1.24E-2</v>
       </c>
       <c r="D4" s="8">
-        <v>0.79090000000000005</v>
+        <v>0.77500000000000002</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1086,13 +1029,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="C5" s="6">
-        <v>1.0500000000000001E-2</v>
+        <v>1.11E-2</v>
       </c>
       <c r="D5" s="8">
-        <v>-0.86860000000000004</v>
+        <v>0.109</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1100,13 +1043,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="C6" s="6">
-        <v>1.04E-2</v>
+        <v>1.0699999999999999E-2</v>
       </c>
       <c r="D6" s="8">
-        <v>0.1046</v>
+        <v>-0.16800000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1114,13 +1057,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="C7" s="6">
-        <v>1.03E-2</v>
+        <v>1.01E-2</v>
       </c>
       <c r="D7" s="8">
-        <v>-0.17929999999999999</v>
+        <v>0.42330000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1128,13 +1071,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C8" s="6">
-        <v>9.7000000000000003E-3</v>
+        <v>9.5999999999999992E-3</v>
       </c>
       <c r="D8" s="8">
-        <v>0.432</v>
+        <v>-0.8841</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1142,13 +1085,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C9" s="6">
-        <v>8.8999999999999999E-3</v>
+        <v>9.4999999999999998E-3</v>
       </c>
       <c r="D9" s="8">
-        <v>0.8</v>
+        <v>0.8085</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1156,13 +1099,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="C10" s="6">
-        <v>8.8000000000000005E-3</v>
+        <v>8.5000000000000006E-3</v>
       </c>
       <c r="D10" s="8">
-        <v>-0.8488</v>
+        <v>0.60719999999999996</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -1170,13 +1113,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="C11" s="6">
-        <v>7.7999999999999996E-3</v>
+        <v>7.4999999999999997E-3</v>
       </c>
       <c r="D11" s="8">
-        <v>0.57599999999999996</v>
+        <v>0.6542</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -1184,13 +1127,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C12" s="6">
-        <v>7.6E-3</v>
+        <v>7.4000000000000003E-3</v>
       </c>
       <c r="D12" s="8">
-        <v>0.65700000000000003</v>
+        <v>0.44429999999999997</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -1198,13 +1141,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C13" s="6">
-        <v>7.1999999999999998E-3</v>
+        <v>7.4000000000000003E-3</v>
       </c>
       <c r="D13" s="8">
-        <v>0.31580000000000003</v>
+        <v>0.27910000000000001</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -1212,13 +1155,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C14" s="6">
-        <v>6.7000000000000002E-3</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="D14" s="8">
-        <v>0.27089999999999997</v>
+        <v>-0.88460000000000005</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -1226,13 +1169,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C15" s="6">
-        <v>6.7000000000000002E-3</v>
+        <v>6.3E-3</v>
       </c>
       <c r="D15" s="8">
-        <v>0.45250000000000001</v>
+        <v>0.61770000000000003</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -1240,13 +1183,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C16" s="6">
-        <v>6.4999999999999997E-3</v>
+        <v>6.1999999999999998E-3</v>
       </c>
       <c r="D16" s="8">
-        <v>0.60099999999999998</v>
+        <v>0.2036</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -1254,13 +1197,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C17" s="6">
-        <v>6.1999999999999998E-3</v>
+        <v>5.8999999999999999E-3</v>
       </c>
       <c r="D17" s="8">
-        <v>-0.1943</v>
+        <v>-0.1875</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -1268,13 +1211,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="C18" s="6">
-        <v>6.0000000000000001E-3</v>
+        <v>5.8999999999999999E-3</v>
       </c>
       <c r="D18" s="8">
-        <v>0.53459999999999996</v>
+        <v>0.17599999999999999</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -1282,13 +1225,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C19" s="6">
-        <v>5.7999999999999996E-3</v>
+        <v>5.4999999999999997E-3</v>
       </c>
       <c r="D19" s="8">
-        <v>0.19189999999999999</v>
+        <v>0.38929999999999998</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -1296,13 +1239,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="C20" s="6">
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="D20" s="8">
-        <v>0.376</v>
+        <v>9.0399999999999994E-2</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -1310,13 +1253,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C21" s="6">
-        <v>5.1999999999999998E-3</v>
+        <v>5.4000000000000003E-3</v>
       </c>
       <c r="D21" s="8">
-        <v>0.27839999999999998</v>
+        <v>0.29220000000000002</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -1324,13 +1267,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="C22" s="6">
-        <v>4.7000000000000002E-3</v>
+        <v>5.3E-3</v>
       </c>
       <c r="D22" s="8">
-        <v>7.9899999999999999E-2</v>
+        <v>0.45960000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -1338,13 +1281,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C23" s="6">
         <v>4.4000000000000003E-3</v>
       </c>
       <c r="D23" s="8">
-        <v>5.6000000000000001E-2</v>
+        <v>9.5600000000000004E-2</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -1352,13 +1295,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="C24" s="6">
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="D24" s="8">
-        <v>0.6643</v>
+        <v>0.76129999999999998</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -1366,13 +1309,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C25" s="6">
-        <v>3.3999999999999998E-3</v>
+        <v>3.5000000000000001E-3</v>
       </c>
       <c r="D25" s="8">
-        <v>0.60040000000000004</v>
+        <v>0.59599999999999997</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -1380,13 +1323,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="C26" s="6">
         <v>3.2000000000000002E-3</v>
       </c>
       <c r="D26" s="8">
-        <v>0.71560000000000001</v>
+        <v>0.55779999999999996</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -1394,13 +1337,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="C27" s="6">
-        <v>2.8999999999999998E-3</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="D27" s="8">
-        <v>-0.66010000000000002</v>
+        <v>0.4269</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -1408,13 +1351,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="C28" s="6">
-        <v>2.7000000000000001E-3</v>
+        <v>1.9E-3</v>
       </c>
       <c r="D28" s="8">
-        <v>0.41299999999999998</v>
+        <v>0.24229999999999999</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -1422,13 +1365,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C29" s="6">
-        <v>1.9E-3</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="D29" s="8">
-        <v>0.41980000000000001</v>
+        <v>0.8679</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -1436,13 +1379,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C30" s="6">
-        <v>1.2999999999999999E-3</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="D30" s="8">
-        <v>-0.28710000000000002</v>
+        <v>-0.50829999999999997</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -1450,13 +1393,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="C31" s="6">
-        <v>1.1000000000000001E-3</v>
+        <v>1E-3</v>
       </c>
       <c r="D31" s="8">
-        <v>-0.48780000000000001</v>
+        <v>-0.35820000000000002</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -1464,13 +1407,13 @@
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>48</v>
+        <v>76</v>
       </c>
       <c r="C32" s="6">
-        <v>8.0000000000000004E-4</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="D32" s="8">
-        <v>-0.84489999999999998</v>
+        <v>-0.51219999999999999</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -1478,13 +1421,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C33" s="6">
-        <v>8.0000000000000004E-4</v>
+        <v>1E-4</v>
       </c>
       <c r="D33" s="8">
-        <v>0.83360000000000001</v>
+        <v>0.19719999999999999</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -1492,41 +1435,13 @@
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="C34" s="6">
-        <v>2.0000000000000001E-4</v>
+        <v>0</v>
       </c>
       <c r="D34" s="8">
-        <v>-0.47920000000000001</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4">
-      <c r="A35" s="1">
-        <v>34</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C35" s="6">
-        <v>1E-4</v>
-      </c>
-      <c r="D35" s="8">
-        <v>0.45700000000000002</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4">
-      <c r="A36" s="1">
-        <v>35</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C36" s="6">
-        <v>0</v>
-      </c>
-      <c r="D36" s="8">
-        <v>3.5000000000000001E-3</v>
+        <v>0.1416</v>
       </c>
     </row>
   </sheetData>
@@ -1537,7 +1452,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D809E70-26AF-C649-8505-80A489EF9743}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="34.1640625" customWidth="1"/>
@@ -1551,10 +1466,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="4" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>30</v>
@@ -1565,16 +1480,16 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B3" s="4">
         <v>2</v>
       </c>
-      <c r="C3" s="6">
-        <v>1.44E-2</v>
-      </c>
-      <c r="D3" s="7">
-        <v>0.91449999999999998</v>
+      <c r="C3" s="1">
+        <v>1.77E-2</v>
+      </c>
+      <c r="D3" s="16">
+        <v>0.92230000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1582,111 +1497,83 @@
         <v>1</v>
       </c>
       <c r="B4" s="4">
-        <v>4</v>
-      </c>
-      <c r="C4" s="6">
-        <v>1.0500000000000001E-2</v>
-      </c>
-      <c r="D4" s="7">
-        <v>-0.86860000000000004</v>
+        <v>7</v>
+      </c>
+      <c r="C4" s="1">
+        <v>9.5999999999999992E-3</v>
+      </c>
+      <c r="D4" s="16">
+        <v>-0.8841</v>
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="4">
-        <v>9</v>
-      </c>
-      <c r="C5" s="6">
-        <v>8.8000000000000005E-3</v>
-      </c>
-      <c r="D5" s="7">
-        <v>-0.8488</v>
+      <c r="A5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="1">
+        <v>13</v>
+      </c>
+      <c r="C5" s="1">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="D5" s="1">
+        <v>-0.88460000000000005</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
-        <v>37</v>
+        <v>86</v>
       </c>
       <c r="B6" s="1">
-        <v>25</v>
-      </c>
-      <c r="C6" s="6">
-        <v>3.2000000000000002E-3</v>
-      </c>
-      <c r="D6" s="8">
-        <v>0.71560000000000001</v>
+        <v>23</v>
+      </c>
+      <c r="C6" s="1">
+        <v>4.1000000000000003E-3</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0.76129999999999998</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B7" s="1">
-        <v>26</v>
-      </c>
-      <c r="C7" s="6">
-        <v>2.8999999999999998E-3</v>
-      </c>
-      <c r="D7" s="8">
-        <v>-0.66010000000000002</v>
+        <v>27</v>
+      </c>
+      <c r="C7" s="1">
+        <v>1.9E-3</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.24229999999999999</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="1" t="s">
-        <v>33</v>
+        <v>87</v>
       </c>
       <c r="B8" s="1">
         <v>28</v>
       </c>
-      <c r="C8" s="6">
-        <v>1.9E-3</v>
-      </c>
-      <c r="D8" s="8">
-        <v>0.41980000000000001</v>
+      <c r="C8" s="1">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.8679</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
-        <v>32</v>
+        <v>77</v>
       </c>
       <c r="B9" s="1">
         <v>31</v>
       </c>
-      <c r="C9" s="6">
-        <v>8.0000000000000004E-4</v>
-      </c>
-      <c r="D9" s="8">
-        <v>-0.84489999999999998</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B10" s="1">
-        <v>32</v>
-      </c>
-      <c r="C10" s="6">
-        <v>8.0000000000000004E-4</v>
-      </c>
-      <c r="D10" s="8">
-        <v>0.83360000000000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B11" s="1">
-        <v>33</v>
-      </c>
-      <c r="C11" s="6">
-        <v>2.0000000000000001E-4</v>
-      </c>
-      <c r="D11" s="8">
-        <v>-0.47920000000000001</v>
+      <c r="C9" s="1">
+        <v>2.9999999999999997E-4</v>
+      </c>
+      <c r="D9" s="1">
+        <v>-0.51219999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1702,20 +1589,20 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="29.33203125" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="2" max="2" width="16.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="4" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>30</v>
@@ -1731,81 +1618,81 @@
       <c r="B3" s="4">
         <v>3</v>
       </c>
-      <c r="C3" s="6">
-        <v>1.21E-2</v>
-      </c>
-      <c r="D3" s="7">
-        <v>0.79090000000000005</v>
+      <c r="C3" s="1">
+        <v>1.24E-2</v>
+      </c>
+      <c r="D3" s="16">
+        <v>0.77500000000000002</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B4" s="4">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1">
+        <v>8.5000000000000006E-3</v>
+      </c>
+      <c r="D4" s="16">
+        <v>0.60719999999999996</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="4">
         <v>10</v>
       </c>
-      <c r="C4" s="6">
-        <v>7.7999999999999996E-3</v>
-      </c>
-      <c r="D4" s="7">
-        <v>0.57599999999999996</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="9">
+      <c r="C5" s="1">
+        <v>7.4999999999999997E-3</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.6542</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="1">
         <v>11</v>
       </c>
-      <c r="C5" s="12">
-        <v>7.6E-3</v>
-      </c>
-      <c r="D5" s="10">
-        <v>0.65700000000000003</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="9">
+      <c r="C6" s="1">
+        <v>7.4000000000000003E-3</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0.44429999999999997</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="1">
         <v>12</v>
       </c>
-      <c r="C6" s="12">
-        <v>7.1999999999999998E-3</v>
-      </c>
-      <c r="D6" s="10">
-        <v>0.31580000000000003</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B7" s="9">
-        <v>14</v>
-      </c>
-      <c r="C7" s="12">
-        <v>6.7000000000000002E-3</v>
-      </c>
-      <c r="D7" s="13">
-        <v>0.45250000000000001</v>
+      <c r="C7" s="1">
+        <v>7.4000000000000003E-3</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.27910000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B8" s="1">
-        <v>15</v>
-      </c>
-      <c r="C8" s="6">
-        <v>6.4999999999999997E-3</v>
-      </c>
-      <c r="D8" s="8">
-        <v>0.60099999999999998</v>
+        <v>14</v>
+      </c>
+      <c r="C8" s="1">
+        <v>6.3E-3</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.61770000000000003</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1813,41 +1700,41 @@
         <v>20</v>
       </c>
       <c r="B9" s="1">
-        <v>18</v>
-      </c>
-      <c r="C9" s="6">
-        <v>5.7999999999999996E-3</v>
-      </c>
-      <c r="D9" s="8">
-        <v>0.19189999999999999</v>
+        <v>15</v>
+      </c>
+      <c r="C9" s="1">
+        <v>6.1999999999999998E-3</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.2036</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B10" s="1">
-        <v>19</v>
-      </c>
-      <c r="C10" s="6">
+        <v>18</v>
+      </c>
+      <c r="C10" s="1">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="D10" s="8">
-        <v>0.376</v>
+      <c r="D10" s="1">
+        <v>0.38929999999999998</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B11" s="1">
-        <v>21</v>
-      </c>
-      <c r="C11" s="6">
-        <v>4.7000000000000002E-3</v>
-      </c>
-      <c r="D11" s="8">
-        <v>7.9899999999999999E-2</v>
+        <v>19</v>
+      </c>
+      <c r="C11" s="1">
+        <v>5.4999999999999997E-3</v>
+      </c>
+      <c r="D11" s="1">
+        <v>9.0399999999999994E-2</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -1855,13 +1742,13 @@
         <v>22</v>
       </c>
       <c r="B12" s="1">
-        <v>23</v>
-      </c>
-      <c r="C12" s="6">
-        <v>4.1000000000000003E-3</v>
-      </c>
-      <c r="D12" s="8">
-        <v>0.6643</v>
+        <v>25</v>
+      </c>
+      <c r="C12" s="1">
+        <v>3.2000000000000002E-3</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0.55779999999999996</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -1869,13 +1756,13 @@
         <v>21</v>
       </c>
       <c r="B13" s="1">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C13" s="1">
-        <v>1.2999999999999999E-3</v>
-      </c>
-      <c r="D13" s="8">
-        <v>-0.28710000000000002</v>
+        <v>1E-3</v>
+      </c>
+      <c r="D13" s="1">
+        <v>-0.35820000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -1896,15 +1783,15 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="4" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>30</v>
@@ -1920,11 +1807,11 @@
       <c r="B3" s="4">
         <v>1</v>
       </c>
-      <c r="C3" s="6">
-        <v>1.9800000000000002E-2</v>
-      </c>
-      <c r="D3" s="7">
-        <v>-0.67190000000000005</v>
+      <c r="C3" s="1">
+        <v>2.12E-2</v>
+      </c>
+      <c r="D3" s="16">
+        <v>-0.6744</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1932,13 +1819,13 @@
         <v>11</v>
       </c>
       <c r="B4" s="4">
-        <v>5</v>
-      </c>
-      <c r="C4" s="6">
-        <v>1.04E-2</v>
-      </c>
-      <c r="D4" s="8">
-        <v>0.1046</v>
+        <v>4</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1.11E-2</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0.109</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1946,13 +1833,13 @@
         <v>10</v>
       </c>
       <c r="B5" s="4">
-        <v>6</v>
-      </c>
-      <c r="C5" s="12">
-        <v>1.03E-2</v>
-      </c>
-      <c r="D5" s="13">
-        <v>-0.17929999999999999</v>
+        <v>5</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1.0699999999999999E-2</v>
+      </c>
+      <c r="D5" s="1">
+        <v>-0.16800000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1962,53 +1849,53 @@
       <c r="B6" s="4">
         <v>8</v>
       </c>
-      <c r="C6" s="12">
-        <v>8.8999999999999999E-3</v>
-      </c>
-      <c r="D6" s="13">
-        <v>0.8</v>
+      <c r="C6" s="1">
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="D6" s="16">
+        <v>0.8085</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="9">
-        <v>13</v>
-      </c>
-      <c r="C7" s="6">
-        <v>6.7000000000000002E-3</v>
-      </c>
-      <c r="D7" s="8">
-        <v>0.27089999999999997</v>
+      <c r="B7" s="1">
+        <v>17</v>
+      </c>
+      <c r="C7" s="1">
+        <v>5.8999999999999999E-3</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.17599999999999999</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B8" s="1">
-        <v>17</v>
-      </c>
-      <c r="C8" s="6">
-        <v>6.0000000000000001E-3</v>
-      </c>
-      <c r="D8" s="8">
-        <v>0.53459999999999996</v>
+        <v>20</v>
+      </c>
+      <c r="C8" s="1">
+        <v>5.4000000000000003E-3</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.29220000000000002</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B9" s="1">
-        <v>20</v>
-      </c>
-      <c r="C9" s="6">
-        <v>5.1999999999999998E-3</v>
-      </c>
-      <c r="D9" s="8">
-        <v>0.27839999999999998</v>
+        <v>21</v>
+      </c>
+      <c r="C9" s="1">
+        <v>5.3E-3</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.45960000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2018,11 +1905,11 @@
       <c r="B10" s="1">
         <v>24</v>
       </c>
-      <c r="C10" s="6">
-        <v>3.3999999999999998E-3</v>
-      </c>
-      <c r="D10" s="8">
-        <v>0.60040000000000004</v>
+      <c r="C10" s="1">
+        <v>3.5000000000000001E-3</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.59599999999999997</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2030,13 +1917,13 @@
         <v>13</v>
       </c>
       <c r="B11" s="1">
-        <v>27</v>
-      </c>
-      <c r="C11" s="6">
-        <v>2.7000000000000001E-3</v>
-      </c>
-      <c r="D11" s="8">
-        <v>0.41299999999999998</v>
+        <v>26</v>
+      </c>
+      <c r="C11" s="1">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.4269</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2044,13 +1931,13 @@
         <v>14</v>
       </c>
       <c r="B12" s="1">
-        <v>30</v>
-      </c>
-      <c r="C12" s="6">
+        <v>29</v>
+      </c>
+      <c r="C12" s="1">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="D12" s="8">
-        <v>-0.48780000000000001</v>
+      <c r="D12" s="1">
+        <v>-0.50829999999999997</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2058,13 +1945,13 @@
         <v>7</v>
       </c>
       <c r="B13" s="1">
-        <v>34</v>
-      </c>
-      <c r="C13" s="6">
+        <v>32</v>
+      </c>
+      <c r="C13" s="1">
         <v>1E-4</v>
       </c>
-      <c r="D13" s="8">
-        <v>0.45700000000000002</v>
+      <c r="D13" s="1">
+        <v>0.19719999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -2072,13 +1959,13 @@
         <v>8</v>
       </c>
       <c r="B14" s="1">
-        <v>35</v>
-      </c>
-      <c r="C14" s="6">
+        <v>33</v>
+      </c>
+      <c r="C14" s="1">
         <v>0</v>
       </c>
-      <c r="D14" s="8">
-        <v>3.5000000000000001E-3</v>
+      <c r="D14" s="1">
+        <v>0.1416</v>
       </c>
     </row>
   </sheetData>
@@ -2099,15 +1986,15 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="4" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>30</v>
@@ -2121,13 +2008,13 @@
         <v>3</v>
       </c>
       <c r="B3" s="4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" s="6">
-        <v>9.7000000000000003E-3</v>
+        <v>1.01E-2</v>
       </c>
       <c r="D3" s="7">
-        <v>0.432</v>
+        <v>0.42330000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2138,10 +2025,10 @@
         <v>16</v>
       </c>
       <c r="C4" s="6">
-        <v>6.1999999999999998E-3</v>
-      </c>
-      <c r="D4" s="13">
-        <v>-0.1943</v>
+        <v>5.8999999999999999E-3</v>
+      </c>
+      <c r="D4" s="11">
+        <v>-0.1875</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2155,7 +2042,7 @@
         <v>4.4000000000000003E-3</v>
       </c>
       <c r="D5" s="8">
-        <v>5.6000000000000001E-2</v>
+        <v>9.5600000000000004E-2</v>
       </c>
     </row>
   </sheetData>
@@ -2177,195 +2064,195 @@
   <sheetData>
     <row r="1" spans="1:4" ht="34">
       <c r="A1" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>87</v>
+        <v>74</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>79</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="D1" s="14" t="s">
-        <v>89</v>
+        <v>80</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="17" t="s">
-        <v>92</v>
-      </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
+      <c r="A2" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="2">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2">
+        <v>1.77E-2</v>
+      </c>
+      <c r="D3" s="13">
+        <v>0.92230000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="17">
+        <v>7</v>
+      </c>
+      <c r="C4" s="17">
+        <v>9.5999999999999992E-3</v>
+      </c>
+      <c r="D4" s="18">
+        <v>-0.8841</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="17">
+        <v>6</v>
+      </c>
+      <c r="C6" s="17">
+        <v>1.01E-2</v>
+      </c>
+      <c r="D6" s="18">
+        <v>0.42330000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B8" s="17">
         <v>1</v>
       </c>
-      <c r="C3" s="2">
-        <v>1.9800000000000002E-2</v>
-      </c>
-      <c r="D3" s="15">
-        <v>-0.67190000000000005</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="2">
-        <v>5</v>
-      </c>
-      <c r="C4" s="2">
-        <v>1.04E-2</v>
-      </c>
-      <c r="D4" s="15">
-        <v>0.1046</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="2">
-        <v>6</v>
-      </c>
-      <c r="C5" s="2">
-        <v>1.03E-2</v>
-      </c>
-      <c r="D5" s="15">
-        <v>-0.17929999999999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B6" s="2">
-        <v>8</v>
-      </c>
-      <c r="C6" s="2">
-        <v>8.8999999999999999E-3</v>
-      </c>
-      <c r="D6" s="15">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="2">
-        <v>3</v>
-      </c>
-      <c r="C8" s="2">
-        <v>1.21E-2</v>
-      </c>
-      <c r="D8" s="15">
-        <v>0.79090000000000005</v>
+      <c r="C8" s="17">
+        <v>2.12E-2</v>
+      </c>
+      <c r="D8" s="18">
+        <v>-0.6744</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2" t="s">
-        <v>44</v>
+        <v>11</v>
       </c>
       <c r="B9" s="2">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C9" s="2">
-        <v>7.7999999999999996E-3</v>
-      </c>
-      <c r="D9" s="15">
-        <v>0.57599999999999996</v>
+        <v>1.11E-2</v>
+      </c>
+      <c r="D9" s="13">
+        <v>0.109</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
+        <v>10</v>
+      </c>
+      <c r="B10" s="17">
+        <v>5</v>
+      </c>
+      <c r="C10" s="17">
+        <v>1.0699999999999999E-2</v>
+      </c>
+      <c r="D10" s="18">
+        <v>-0.16800000000000001</v>
+      </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="B11" s="2">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C11" s="2">
-        <v>1.44E-2</v>
-      </c>
-      <c r="D11" s="15">
-        <v>0.91449999999999998</v>
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="D11" s="13">
+        <v>0.8085</v>
       </c>
     </row>
     <row r="12" spans="1:4">
-      <c r="A12" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B12" s="2">
-        <v>4</v>
-      </c>
-      <c r="C12" s="2">
-        <v>1.0500000000000001E-2</v>
-      </c>
-      <c r="D12" s="15">
-        <v>-0.86860000000000004</v>
-      </c>
+      <c r="A12" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
     </row>
     <row r="13" spans="1:4">
-      <c r="A13" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B13" s="2">
+      <c r="A13" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="17">
+        <v>3</v>
+      </c>
+      <c r="C13" s="17">
+        <v>1.24E-2</v>
+      </c>
+      <c r="D13" s="18">
+        <v>0.77500000000000002</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="2">
         <v>9</v>
       </c>
-      <c r="C13" s="2">
-        <v>8.8000000000000005E-3</v>
-      </c>
-      <c r="D13" s="15">
-        <v>-0.8488</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
+      <c r="C14" s="2">
+        <v>8.5000000000000006E-3</v>
+      </c>
+      <c r="D14" s="13">
+        <v>0.60719999999999996</v>
+      </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2" t="s">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="B15" s="2">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C15" s="2">
-        <v>9.7000000000000003E-3</v>
-      </c>
-      <c r="D15" s="15">
-        <v>0.432</v>
+        <v>7.4999999999999997E-3</v>
+      </c>
+      <c r="D15" s="13">
+        <v>0.6542</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A5:D5"/>
     <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>